<commit_message>
feat(masterdata): Dodge 모드(9)·맵(8) 추가, 두 큐에 허용
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/table/Datas/#GameMode.xlsx
+++ b/table/Datas/#GameMode.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -783,6 +783,37 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="B13" t="n">
+        <v>9</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Dodge</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>피하기</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>스테이지마다 바뀌는 위험을 끝까지 피하는 생존전</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>2</v>
+      </c>
+      <c r="G13" t="n">
+        <v>8</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Assets/Scenes/Dodge.unity</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(masterdata): MountedArchery 모드(10)·맵(14)·설정 표, 일반 큐 허용
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/table/Datas/#GameMode.xlsx
+++ b/table/Datas/#GameMode.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -814,6 +814,32 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="B14" t="n">
+        <v>10</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>MountedArchery</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>말 위 활쏘기</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>1</v>
+      </c>
+      <c r="G14" t="n">
+        <v>8</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Assets/Scenes/MountedArchery.unity</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>